<commit_message>
Add Data Insights tab: quantitative analysis of all 382 winning emails
</commit_message>
<xml_diff>
--- a/Qualtrics_Email_Framework_Playbook.xlsx
+++ b/Qualtrics_Email_Framework_Playbook.xlsx
@@ -8,22 +8,23 @@
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Frameworks" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Body Principles" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Email Templates" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Subject Lines" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Swap-In Banks" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Checklist &amp; Sources" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Winning Emails (382)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Data Insights" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Frameworks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Body Principles" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Email Templates" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Subject Lines" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Swap-In Banks" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Checklist &amp; Sources" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Winning Emails (382)" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Frameworks'!$A$1:$C$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Body Principles'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Email Templates'!$A$1:$F$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Subject Lines'!$A$1:$F$47</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Swap-In Banks'!$A$1:$D$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Checklist &amp; Sources'!$A$1:$B$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Winning Emails (382)'!$A$1:$F$383</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Frameworks'!$A$1:$C$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Body Principles'!$A$1:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Email Templates'!$A$1:$F$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Subject Lines'!$A$1:$F$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Swap-In Banks'!$A$1:$D$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Checklist &amp; Sources'!$A$1:$B$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Winning Emails (382)'!$A$1:$F$383</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -32,7 +33,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,6 +61,19 @@
       <color rgb="002D2A70"/>
       <sz val="11"/>
     </font>
+    <font>
+      <color rgb="00555555"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002D2A70"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -79,7 +93,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -101,11 +115,25 @@
         <color rgb="00DDDDDD"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -131,6 +159,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -496,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -530,96 +570,109 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Frameworks</t>
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Data Insights</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>The 5 proven frameworks, when to use each, and how often they won.</t>
+          <t>Quantitative analysis of all 382 emails: framework distribution, ideal length, tactical pattern prevalence, and the 3 rules from the data.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Body Principles</t>
+          <t>Frameworks</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>The 6 traits shared by nearly every winning email.</t>
+          <t>The 5 proven frameworks, when to use each, and how often they won.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Email Templates</t>
+          <t>Body Principles</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>16 fill-in-the-blank templates, each paired with a REAL meeting-booking example + why it works.</t>
+          <t>The 6 traits shared by nearly every winning email.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Subject Lines</t>
+          <t>Email Templates</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Research-backed rules, per-framework strategies, 28 subject templates, and real examples.</t>
+          <t>16 fill-in-the-blank templates, each paired with a REAL meeting-booking example + why it works.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Swap-In Banks</t>
+          <t>Subject Lines</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Mix-and-match openers, peer-proof by industry, value lines, and CTAs ranked by frequency.</t>
+          <t>Research-backed rules, per-framework strategies, 28 subject templates, and real examples.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Checklist &amp; Sources</t>
+          <t>Swap-In Banks</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Pre-send checklist + cited research sources.</t>
+          <t>Mix-and-match openers, peer-proof by industry, value lines, and CTAs ranked by frequency.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
+          <t>Checklist &amp; Sources</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Pre-send checklist + cited research sources.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
           <t>Winning Emails (382)</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Every source email that booked a meeting, categorized — filter by Framework or Industry.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="78" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
+    <row r="13" ht="78" customHeight="1"/>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>HOW TO USE</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>1) Pick your scenario in 'Frameworks'.  2) Grab the matching template in 'Email Templates' and model your fill-ins on the real example beneath it.  3) Pick a subject line.  4) Remix with 'Swap-In Banks' (peer proof for your industry + a CTA).  5) Run the 'Checklist' before sending.  Tip: in any tab, click the header row &gt; Data &gt; Create a filter to slice by Framework or Industry.</t>
         </is>
@@ -631,6 +684,657 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Data Insights: What the 382 Winning Emails Have in Common</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Quantitative analysis of all 382 categorized emails — structural patterns of the winning set. Note: no reply/meeting labels exist in the data, so these are prevalence patterns, not outcome-weighted win rates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>1. FRAMEWORK DISTRIBUTION — what reps reach for</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Share</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Takeaway</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>F3 — Role + Peer Proof (Cold)</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="n">
+        <v>135</v>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>35%</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>The workhorse: most-used play for pure cold outreach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>F4 — Trigger Strike (Intent/Signal)</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="n">
+        <v>71</v>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>19%</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>Most disciplined cohort — see section 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>F1 — You Already Use Us (Expansion)</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>61</v>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Expansion into existing accounts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>F2 — Reconnect / New POC</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>Shortest emails in the set (93 words avg).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>F5 — Borrowed Trust (Referral/On-site)</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="n">
+        <v>55</v>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>14%</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Highest peer-proof rate (51%), softest CTA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>2. LENGTH — winners are short and disciplined</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr"/>
+      <c r="D13" s="13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Median body length</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>100 words</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr"/>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>63% of all emails land between 60–119 words.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>Mean body length</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>103 words</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr"/>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>Only 9% exceed 150 words — the "wall of text" is absent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Median subject length</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>3 words / 27 chars</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr"/>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>Mobile-preview safe. Mean: 3.7 words / 29 chars.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>3. SUBJECT LINES — relational, not salesy</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>Top keywords</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>partnership, alignment, intro, welcome, initiatives, experience, insights — conversation-openers, not pitch words. "Demo", "solution", and "save" barely appear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Rule of thumb</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Keep it ≤3 words. The subject sets up a conversation, not a pitch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>4. TACTICAL PATTERN PREVALENCE — across all 382</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Tactic</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>% of emails</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr"/>
+      <c r="D23" s="13" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>Personalized first line (name + role/company ref)</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>79%</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr"/>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>Near-universal baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>Value/relevance-first opening move</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>49%</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr"/>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>Beats self-intro openers (35%) — lead with relevance, not your title.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>Soft availability framing ("next couple weeks")</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>45%</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr"/>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>Lowers commitment friction on the ask.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>Direct time ask (15/20/30-min, calendar)</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>41%</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr"/>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>Roughly tied with soft question CTAs — both pull weight.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>Soft question CTA ("open to…", "worth…?")</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>38%</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr"/>
+      <c r="D28" s="14" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>Specific 15/20/30-minute ask</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>36%</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr"/>
+      <c r="D29" s="14" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>Social/peer-proof language ("teams at…", "companies like…")</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>35%</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr"/>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>The dominant trust device in the set.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>References a trigger/event</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>34%</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr"/>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t>News, new role, launch, initiative, earnings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>Names a specific company/org as proof</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>27%</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="inlineStr"/>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>Named peers &gt; generic claims.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>Quantified stats ($ / % / ROI)</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>4–8%</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr"/>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>Strikingly rare. Credibility comes from "who we help", not numbers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>5. PER-FRAMEWORK BREAKDOWN — F4 (Trigger Strike) is the standout</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Avg words</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>Peer proof</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>Key traits</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t>F1 — You Already Use Us</t>
+        </is>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>109</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>43%</t>
+        </is>
+      </c>
+      <c r="D37" s="14" t="inlineStr">
+        <is>
+          <t>Soft CTA-heavy (46%); leans on existing relationship.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>F2 — Reconnect / New POC</t>
+        </is>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="inlineStr">
+        <is>
+          <t>Shortest; relies on prior context instead of proof.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>F3 — Role + Peer Proof</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>106</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>27%</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="inlineStr">
+        <is>
+          <t>Highest volume; balanced CTA mix (39% soft / 40% time-ask).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>F4 — Trigger Strike</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
+      <c r="C40" s="14" t="inlineStr">
+        <is>
+          <t>45%</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr">
+        <is>
+          <t>BEST-IN-CLASS: 77% reference a trigger, 54% use outcome/value verbs, 48% make a specific time ask — shorter, more specific, harder-closing all at once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>F5 — Borrowed Trust</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>51%</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>Highest peer proof; softest close (29% direct ask) — the warm intro carries it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>6. THREE RULES FROM THE DATA</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="15" t="inlineStr">
+        <is>
+          <t>Rule 1 — Keep it tight</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>~100 words body, ≤3-word subject. The winners are disciplined about length on both ends.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="15" t="inlineStr">
+        <is>
+          <t>Rule 2 — Lead with relevance + a named peer, not your title</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>"Teams like [peer] are doing X" outperforms "My name is… I work on…" and beats stat-dumping, which barely appears in winning emails.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="15" t="inlineStr">
+        <is>
+          <t>Rule 3 — Anchor on a trigger whenever one exists</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Trigger-based emails (F4) are the tightest, most value-dense, hardest-closing cohort in the entire set. Model cold outreach on F4's structure.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B20:D20"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -752,7 +1456,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -855,7 +1559,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1949,7 +2653,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3160,7 +3864,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3759,7 +4463,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3934,7 +4638,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>